<commit_message>
Supplementary: remove duplicated and withdrawn material, renumber to 11 tables and 5 figures
</commit_message>
<xml_diff>
--- a/Source_Data.xlsx
+++ b/Source_Data.xlsx
@@ -28,8 +28,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FigS4a" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FigS4b" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FigS5" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FigS6" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FigS7" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -715,30 +713,6 @@
       <c r="B22" t="inlineStr">
         <is>
           <t>OIS bands at 24.9060 and 27.2367 (permutation P 0.0, 1000 permutations, bootstrap 95% for the cuts 24.41 to 25.36 and 27.12 to 28.76).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>FigS6</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Delta C by group and the difference of differences.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>FigS7</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>CSF alpha-synuclein SAA positivity with Wilson 95% CI.</t>
         </is>
       </c>
     </row>
@@ -17195,446 +17169,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>stratum</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>events</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>dC</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>lo</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Hyposmia</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1003</v>
-      </c>
-      <c r="C2" t="n">
-        <v>68</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.1367511105775003</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.07176303406546798</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.2033499504888623</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>hyposmia + DAT deficit</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>265</v>
-      </c>
-      <c r="C3" t="n">
-        <v>46</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.1147967752771246</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.01459391538041605</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.213245069502198</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.022</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>hyposmia + no DAT deficit</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>738</v>
-      </c>
-      <c r="C4" t="n">
-        <v>22</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.02938948644144834</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-0.08428725707340748</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.1379696194166478</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.516</v>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>RBD and variant-carrier</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>756</v>
-      </c>
-      <c r="C5" t="n">
-        <v>84</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.06663608638516272</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.000298421580499159</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.1339458556428066</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>difference between groups</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>0.07011502419233762</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>ci_lower</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>-0.03219555379416288</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>ci_upper</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>0.1677101189620693</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>0.181</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>n_boot</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="31" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>group</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>positive</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>rate_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>wilson_ci_lower_pct</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>wilson_ci_upper_pct</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>GBA1</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>56</v>
-      </c>
-      <c r="C2" t="n">
-        <v>52</v>
-      </c>
-      <c r="D2" t="n">
-        <v>92.85714285714286</v>
-      </c>
-      <c r="E2" t="n">
-        <v>83.02455193613837</v>
-      </c>
-      <c r="F2" t="n">
-        <v>97.18739634269382</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LRRK2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>126</v>
-      </c>
-      <c r="C3" t="n">
-        <v>84</v>
-      </c>
-      <c r="D3" t="n">
-        <v>66.66666666666666</v>
-      </c>
-      <c r="E3" t="n">
-        <v>58.050191549565</v>
-      </c>
-      <c r="F3" t="n">
-        <v>74.29694963391255</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sporadic</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>824</v>
-      </c>
-      <c r="C4" t="n">
-        <v>764</v>
-      </c>
-      <c r="D4" t="n">
-        <v>92.71844660194175</v>
-      </c>
-      <c r="E4" t="n">
-        <v>90.73916822650787</v>
-      </c>
-      <c r="F4" t="n">
-        <v>94.30126946809052</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Fisher exact P, GBA1 vs LRRK2</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>8.780179984141926e-05</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Label the measured score UPSIT in figures, supplementary and source data
</commit_message>
<xml_diff>
--- a/Source_Data.xlsx
+++ b/Source_Data.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cumulative/dynamic AUC with IPCW, 95% CI from 1,000 bootstrap resamples. The row OIS minus UPSIT total carries the paired P.</t>
+          <t>Cumulative/dynamic AUC with IPCW, 95% CI from 1,000 bootstrap resamples. The row OIS minus UPSIT carries the paired P.</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Delta C (OIS minus UPSIT total) with 95% CI from 1,000 paired bootstrap resamples. P of 0 means below 1/1000.</t>
+          <t>Delta C (OIS minus UPSIT) with 95% CI from 1,000 paired bootstrap resamples. P of 0 means below 1/1000.</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -6057,7 +6057,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -6128,7 +6128,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -6243,7 +6243,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -6314,7 +6314,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -20111,7 +20111,7 @@
   <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -20160,7 +20160,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -20394,7 +20394,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -20451,7 +20451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -20529,7 +20529,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OIS minus UPSIT total</t>
+          <t>OIS minus UPSIT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -20557,7 +20557,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -20635,7 +20635,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OIS minus UPSIT total</t>
+          <t>OIS minus UPSIT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -20663,7 +20663,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -20741,7 +20741,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OIS minus UPSIT total</t>
+          <t>OIS minus UPSIT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -21089,7 +21089,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -21109,7 +21109,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="I8" t="b">
@@ -21355,7 +21355,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -21375,7 +21375,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="I15" t="b">
@@ -21621,7 +21621,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -21641,7 +21641,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>UPSIT total</t>
+          <t>UPSIT</t>
         </is>
       </c>
       <c r="I22" t="b">

</xml_diff>

<commit_message>
Drop the centre split from Supplementary Fig 3 and source data
</commit_message>
<xml_diff>
--- a/Source_Data.xlsx
+++ b/Source_Data.xlsx
@@ -7245,14 +7245,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
@@ -7392,56 +7392,6 @@
       </c>
       <c r="G5" t="n">
         <v>0.001</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Centre split, discovery 5 sites</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>290</v>
-      </c>
-      <c r="C6" t="n">
-        <v>16</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.1107178968655207</v>
-      </c>
-      <c r="E6" t="n">
-        <v>-0.02033881155396369</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.2342383733766689</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.092</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Centre split, external 6 sites</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>343</v>
-      </c>
-      <c r="C7" t="n">
-        <v>17</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.275624301155423</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.1496993785553496</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.4207720105124834</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish corrected JTM analysis and aggregate audit outputs
</commit_message>
<xml_diff>
--- a/Source_Data.xlsx
+++ b/Source_Data.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Delta C (OIS minus UPSIT) with 95% CI from 1,000 paired bootstrap resamples. P of 0 means below 1/1000.</t>
+          <t>Delta C (OIS minus UPSIT) with 95% CI from 1,000 paired bootstrap resamples and two-sided P values with a reporting floor of 0.001. Landmark risk sets retain participants observed event-free beyond the landmark, with follow-up restarted there.</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6430,7 @@
   <cols>
     <col width="59" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -6553,7 +6553,11 @@
       <c r="B4" t="n">
         <v>2441</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>separate correlation branch from n=2453; excludes 12 without measured UPSIT</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
@@ -6574,7 +6578,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>excluded 78</t>
+          <t>survival branch starts at n=2453; excludes 78 prevalent cases</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -7310,13 +7314,13 @@
         <v>0.1367511105775003</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06714499999651713</v>
+        <v>0.07176303406546798</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2038020769712451</v>
+        <v>0.2033499504888623</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="3">
@@ -7326,7 +7330,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>993</v>
+        <v>817</v>
       </c>
       <c r="C3" t="n">
         <v>58</v>
@@ -7335,13 +7339,13 @@
         <v>0.1113560033585222</v>
       </c>
       <c r="E3" t="n">
-        <v>0.04132191162631785</v>
+        <v>0.03826172076048909</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1851760139890274</v>
+        <v>0.178886985322326</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="4">
@@ -7351,7 +7355,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>962</v>
+        <v>432</v>
       </c>
       <c r="C4" t="n">
         <v>27</v>
@@ -7360,13 +7364,13 @@
         <v>0.1563670411985019</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02177772238839035</v>
+        <v>0.02786302584215341</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2746808286296951</v>
+        <v>0.2842896655707283</v>
       </c>
       <c r="G4" t="n">
-        <v>0.024</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="5">
@@ -17363,7 +17367,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -17460,7 +17464,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4785343099794064</v>
+        <v>0.4785351280306384</v>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
@@ -17475,7 +17479,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4370711165066363</v>
+        <v>0.4370719748383699</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
@@ -17490,7 +17494,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5179678830972674</v>
+        <v>0.5179686594550252</v>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
@@ -17505,7 +17509,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6.521609150319231e-81</v>
+        <v>6.516977213043236e-81</v>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
@@ -17520,7 +17524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.9481109075766492</v>
+        <v>0.9481085584953793</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
@@ -17535,7 +17539,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1.309759823861657</v>
+        <v>1.309836981901182</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
@@ -17562,7 +17566,7 @@
         <v>140</v>
       </c>
       <c r="E12" t="n">
-        <v>20.00937027262781</v>
+        <v>20.00933530464462</v>
       </c>
       <c r="F12" t="n">
         <v>20.58571428571429</v>
@@ -17581,7 +17585,7 @@
         <v>140</v>
       </c>
       <c r="E13" t="n">
-        <v>21.48656097751841</v>
+        <v>21.48664368248626</v>
       </c>
       <c r="F13" t="n">
         <v>21.77857142857143</v>
@@ -17600,7 +17604,7 @@
         <v>140</v>
       </c>
       <c r="E14" t="n">
-        <v>22.31261653401205</v>
+        <v>22.31261632474947</v>
       </c>
       <c r="F14" t="n">
         <v>22.85714285714286</v>
@@ -17619,7 +17623,7 @@
         <v>139</v>
       </c>
       <c r="E15" t="n">
-        <v>23.14123595126721</v>
+        <v>23.14117460321857</v>
       </c>
       <c r="F15" t="n">
         <v>23.61151079136691</v>
@@ -17638,7 +17642,7 @@
         <v>140</v>
       </c>
       <c r="E16" t="n">
-        <v>23.88921641549879</v>
+        <v>23.88913706361943</v>
       </c>
       <c r="F16" t="n">
         <v>22.91428571428571</v>
@@ -17657,7 +17661,7 @@
         <v>140</v>
       </c>
       <c r="E17" t="n">
-        <v>24.62586149250055</v>
+        <v>24.62582297801962</v>
       </c>
       <c r="F17" t="n">
         <v>22.83571428571429</v>
@@ -17676,7 +17680,7 @@
         <v>139</v>
       </c>
       <c r="E18" t="n">
-        <v>25.49937204580442</v>
+        <v>25.49920972879455</v>
       </c>
       <c r="F18" t="n">
         <v>24.84172661870504</v>
@@ -17695,7 +17699,7 @@
         <v>140</v>
       </c>
       <c r="E19" t="n">
-        <v>26.82627740677995</v>
+        <v>26.82634735776123</v>
       </c>
       <c r="F19" t="n">
         <v>27.67857142857143</v>
@@ -17714,7 +17718,7 @@
         <v>140</v>
       </c>
       <c r="E20" t="n">
-        <v>29.86639526744555</v>
+        <v>29.86644450816058</v>
       </c>
       <c r="F20" t="n">
         <v>31.37142857142857</v>
@@ -17733,7 +17737,7 @@
         <v>140</v>
       </c>
       <c r="E21" t="n">
-        <v>35.24503481673628</v>
+        <v>35.24502112524028</v>
       </c>
       <c r="F21" t="n">
         <v>34.4</v>
@@ -20824,10 +20828,10 @@
         <v>0.7758884620002401</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6961440671496674</v>
+        <v>0.6904716741353928</v>
       </c>
       <c r="G2" t="n">
-        <v>0.846224344784636</v>
+        <v>0.8482365331554907</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -20862,10 +20866,10 @@
         <v>0.7614059310841638</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6803207214004487</v>
+        <v>0.6740277730288694</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8410861586378321</v>
+        <v>0.8373791713854698</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -20900,10 +20904,10 @@
         <v>0.6818945851842958</v>
       </c>
       <c r="F4" t="n">
-        <v>0.601411596029658</v>
+        <v>0.6032299354425213</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7619669655003286</v>
+        <v>0.7641658762950061</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -20935,13 +20939,13 @@
         <v>68</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7789350462240365</v>
+        <v>0.8124924960979709</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7063766090138057</v>
+        <v>0.7453975386035259</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8456793224439865</v>
+        <v>0.8756579419528743</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -20976,10 +20980,10 @@
         <v>0.8195461640052828</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7481285089828597</v>
+        <v>0.748797476891089</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8790851054777398</v>
+        <v>0.8786339353918812</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -21014,10 +21018,10 @@
         <v>0.8350642334013687</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7699501487971604</v>
+        <v>0.7741060224062686</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8964003644382291</v>
+        <v>0.894507130532964</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -21052,10 +21056,10 @@
         <v>0.6983131228238684</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6323701633374745</v>
+        <v>0.6325314842230595</v>
       </c>
       <c r="G8" t="n">
-        <v>0.7605808158737484</v>
+        <v>0.7601279052264246</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -21090,10 +21094,10 @@
         <v>0.6572892173328855</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5775677633030891</v>
+        <v>0.5719882023092975</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7384148322333722</v>
+        <v>0.7368203737257351</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -21128,10 +21132,10 @@
         <v>0.6550218340611353</v>
       </c>
       <c r="F10" t="n">
-        <v>0.5746951081074859</v>
+        <v>0.5638848904656721</v>
       </c>
       <c r="G10" t="n">
-        <v>0.7343213628996684</v>
+        <v>0.7461789216649146</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -21166,10 +21170,10 @@
         <v>0.598925092374874</v>
       </c>
       <c r="F11" t="n">
-        <v>0.4889751727903909</v>
+        <v>0.4988342291750721</v>
       </c>
       <c r="G11" t="n">
-        <v>0.705595121003485</v>
+        <v>0.7118177210856019</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -21201,13 +21205,13 @@
         <v>46</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6644272757809876</v>
+        <v>0.7232112865300638</v>
       </c>
       <c r="F12" t="n">
-        <v>0.5774427587794394</v>
+        <v>0.627619849729512</v>
       </c>
       <c r="G12" t="n">
-        <v>0.7492222621392767</v>
+        <v>0.806199271087604</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -21242,10 +21246,10 @@
         <v>0.7559623782331206</v>
       </c>
       <c r="F13" t="n">
-        <v>0.670804765928485</v>
+        <v>0.6743027336017332</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8283824579201958</v>
+        <v>0.8312246230417141</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -21280,10 +21284,10 @@
         <v>0.7643600940544172</v>
       </c>
       <c r="F14" t="n">
-        <v>0.6794321146709982</v>
+        <v>0.6763515078893891</v>
       </c>
       <c r="G14" t="n">
-        <v>0.8358201241245602</v>
+        <v>0.8405852416385041</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -21318,10 +21322,10 @@
         <v>0.6495633187772926</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5599876233840836</v>
+        <v>0.5571224773965076</v>
       </c>
       <c r="G15" t="n">
-        <v>0.7341463740948562</v>
+        <v>0.7325541641540069</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -21356,10 +21360,10 @@
         <v>0.5174973488865323</v>
       </c>
       <c r="F16" t="n">
-        <v>0.3568099784863556</v>
+        <v>0.3606151581682794</v>
       </c>
       <c r="G16" t="n">
-        <v>0.7076791489274603</v>
+        <v>0.7186785106291032</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -21394,10 +21398,10 @@
         <v>0.4240266626268747</v>
       </c>
       <c r="F17" t="n">
-        <v>0.2918805967205791</v>
+        <v>0.2758386377721874</v>
       </c>
       <c r="G17" t="n">
-        <v>0.5916960836378793</v>
+        <v>0.5773915407952021</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -21432,10 +21436,10 @@
         <v>0.8112407211028632</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7098441598110434</v>
+        <v>0.7010567370559641</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8975412720155463</v>
+        <v>0.8972053503927702</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -21467,13 +21471,13 @@
         <v>22</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6708074534161491</v>
+        <v>0.7866989850022724</v>
       </c>
       <c r="F19" t="n">
-        <v>0.5600835279054003</v>
+        <v>0.6484275184275183</v>
       </c>
       <c r="G19" t="n">
-        <v>0.7841782884533347</v>
+        <v>0.8904376500193573</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -21508,10 +21512,10 @@
         <v>0.6556582336009695</v>
       </c>
       <c r="F20" t="n">
-        <v>0.4926652445537008</v>
+        <v>0.4993943623106885</v>
       </c>
       <c r="G20" t="n">
-        <v>0.8088717421278977</v>
+        <v>0.8154109024267019</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -21546,10 +21550,10 @@
         <v>0.71898197242842</v>
       </c>
       <c r="F21" t="n">
-        <v>0.5615507865276973</v>
+        <v>0.5668409738846262</v>
       </c>
       <c r="G21" t="n">
-        <v>0.8650031167372969</v>
+        <v>0.8835749616483839</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -21584,10 +21588,10 @@
         <v>0.6895924859869716</v>
       </c>
       <c r="F22" t="n">
-        <v>0.5732069489656791</v>
+        <v>0.5621838670821411</v>
       </c>
       <c r="G22" t="n">
-        <v>0.8033412510630408</v>
+        <v>0.8126556125511423</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>

</xml_diff>